<commit_message>
scan: seg4 2026-06-19 01:21 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-06-18.xlsx
+++ b/output/full_scan/batch_seq5_2026-06-18.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O78"/>
+  <dimension ref="A1:O79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2912,21 +2912,21 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>4912</v>
+        <v>4971</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>聯德控股-KY</t>
+          <t>IET-KY</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>414.9415691648357</v>
+        <v>415.8966667669022</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>88.7</v>
+        <v>578</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>40.48941601852732</v>
+        <v>42.4756909475305</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>21.92526924945886</v>
+        <v>18.18444553509089</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.4642647104162655</v>
+        <v>1.280168853123853</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-1.651751336117441</v>
+        <v>-11.71310080143029</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>4968</v>
+        <v>4912</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>立積</t>
+          <t>聯德控股-KY</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>405.4390491450181</v>
+        <v>414.9415691648357</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>113.5</v>
+        <v>88.7</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>51.64470062649737</v>
+        <v>40.48941601852732</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>15.03810387975169</v>
+        <v>21.92526924945886</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.9436388118154152</v>
+        <v>0.4642647104162655</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.2179854210958549</v>
+        <v>-1.651751336117441</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>4951</v>
+        <v>4968</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>精拓科</t>
+          <t>立積</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>399.3551308337978</v>
+        <v>405.4390491450181</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>98.5</v>
+        <v>113.5</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>38.01272219542637</v>
+        <v>51.64470062649737</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>30.5416879934838</v>
+        <v>15.03810387975169</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.4660293976121147</v>
+        <v>0.9436388118154152</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-2.883960031834654</v>
+        <v>-0.2179854210958549</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>4554</v>
+        <v>4951</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>橙的</t>
+          <t>精拓科</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>397.326829927377</v>
+        <v>399.3551308337978</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>30.15</v>
+        <v>98.5</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.59100748686698</v>
+        <v>38.01272219542637</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>20.01429935429498</v>
+        <v>30.5416879934838</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.5914351126301318</v>
+        <v>0.4660293976121147</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.0687306193457521</v>
+        <v>-2.883960031834654</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>4949</v>
+        <v>4554</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>有成精密</t>
+          <t>橙的</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>393.357469378124</v>
+        <v>397.326829927377</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>88.5</v>
+        <v>30.15</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.15450711094941</v>
+        <v>48.59100748686698</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>19.04907989258658</v>
+        <v>20.01429935429498</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.316417918979208</v>
+        <v>0.5914351126301318</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-1.524525158684565</v>
+        <v>-0.0687306193457521</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>4989</v>
+        <v>4949</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>榮科</t>
+          <t>有成精密</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>385.6928629727696</v>
+        <v>393.357469378124</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>85.5</v>
+        <v>88.5</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>45.36531126681511</v>
+        <v>45.15450711094941</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>23.15948230277193</v>
+        <v>19.04907989258658</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.5782961253706307</v>
+        <v>0.316417918979208</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-1.208606359923476</v>
+        <v>-1.524525158684565</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>5225</v>
+        <v>4989</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>東科-KY</t>
+          <t>榮科</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>384.8270806513195</v>
+        <v>385.6928629727696</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>74</v>
+        <v>85.5</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>51.82327297092611</v>
+        <v>45.36531126681511</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>23.82528789621933</v>
+        <v>23.15948230277193</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.4032416254928237</v>
+        <v>0.5782961253706307</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.3343125273431815</v>
+        <v>-1.208606359923476</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>4582</v>
+        <v>5225</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>聚恆-創</t>
+          <t>東科-KY</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>379.7857835421845</v>
+        <v>384.8270806513195</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>26.55</v>
+        <v>74</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>45.91279110977823</v>
+        <v>51.82327297092611</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>14.12439689766018</v>
+        <v>23.82528789621933</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3654901683459761</v>
+        <v>0.4032416254928237</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>2</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.3212228621953663</v>
+        <v>0.3343125273431815</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>4966</v>
+        <v>4582</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>譜瑞-KY</t>
+          <t>聚恆-創</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>379.7027145711585</v>
+        <v>379.7857835421845</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>693</v>
+        <v>26.55</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>47.15187016779621</v>
+        <v>45.91279110977823</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>20.26464521604339</v>
+        <v>14.12439689766018</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.7809139007535938</v>
+        <v>0.3654901683459761</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-15.15443399626416</v>
+        <v>0.3212228621953663</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>4588</v>
+        <v>4966</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>玖鼎電力</t>
+          <t>譜瑞-KY</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>378.8558614556132</v>
+        <v>379.7027145711585</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>59.1</v>
+        <v>693</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>52.78195114708897</v>
+        <v>47.15187016779621</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>19.30983877241772</v>
+        <v>20.26464521604339</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.2992958575398801</v>
+        <v>0.7809139007535938</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.06879404478219189</v>
+        <v>-15.15443399626416</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4577</v>
+        <v>4588</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>達航科技</t>
+          <t>玖鼎電力</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>368.7906625708485</v>
+        <v>378.8558614556132</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>87.40000000000001</v>
+        <v>59.1</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>31.47076035440847</v>
+        <v>52.78195114708897</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>33.06383611047038</v>
+        <v>19.30983877241772</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.3571824043472644</v>
+        <v>0.2992958575398801</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.5863985012530701</v>
+        <v>0.06879404478219189</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4927</v>
+        <v>4577</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>泰鼎-KY</t>
+          <t>達航科技</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>368.262077291427</v>
+        <v>368.7906625708485</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>51.1</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>48.06059763963739</v>
+        <v>31.47076035440847</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>15.18162563458044</v>
+        <v>33.06383611047038</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.3309459528871115</v>
+        <v>0.3571824043472644</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>1</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.4226341166552263</v>
+        <v>-0.5863985012530701</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>4956</v>
+        <v>4927</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>光鋐</t>
+          <t>泰鼎-KY</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>364.8358801609813</v>
+        <v>368.262077291427</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>38.5</v>
+        <v>51.1</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>40.44601340038991</v>
+        <v>48.06059763963739</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.21769469212498</v>
+        <v>15.18162563458044</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.3171645735819733</v>
+        <v>0.3309459528871115</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.5454464087701214</v>
+        <v>-0.4226341166552263</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>4749</v>
+        <v>4956</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>新應材</t>
+          <t>光鋐</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>358.8370997741439</v>
+        <v>364.8358801609813</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>991</v>
+        <v>38.5</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>48.98243779401277</v>
+        <v>40.44601340038991</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>16.89598169375544</v>
+        <v>20.21769469212498</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.9152259697758472</v>
+        <v>0.3171645735819733</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-8.399572587812521</v>
+        <v>-0.5454464087701214</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>4585</v>
+        <v>4749</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>達明</t>
+          <t>新應材</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>349.0680639776608</v>
+        <v>358.8370997741439</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>313.5</v>
+        <v>991</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>43.70014234521541</v>
+        <v>48.98243779401277</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>21.24361241693884</v>
+        <v>16.89598169375544</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.3278856068631477</v>
+        <v>0.9152259697758472</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-4.23976118091398</v>
+        <v>-8.399572587812521</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>4933</v>
+        <v>4585</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>友輝</t>
+          <t>達明</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>337.9086163104924</v>
+        <v>349.0680639776608</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>67.40000000000001</v>
+        <v>313.5</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>43.86850397644629</v>
+        <v>43.70014234521541</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>22.42273932691763</v>
+        <v>21.24361241693884</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.3753801016283741</v>
+        <v>0.3278856068631477</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.90364445320067</v>
+        <v>-4.23976118091398</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6136</v>
+        <v>4933</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>富爾特</t>
+          <t>友輝</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>331.834297176632</v>
+        <v>337.9086163104924</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>25.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>47.87250034652035</v>
+        <v>43.86850397644629</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>11.63842684672709</v>
+        <v>22.42273932691763</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.5127761157963185</v>
+        <v>0.3753801016283741</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.087572741938302</v>
+        <v>-0.90364445320067</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>5243</v>
+        <v>6136</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>乙盛-KY</t>
+          <t>富爾特</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>328.1511907956772</v>
+        <v>331.834297176632</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>109.5</v>
+        <v>25.3</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>46.8871413451367</v>
+        <v>47.87250034652035</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>15.10854183223336</v>
+        <v>11.63842684672709</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.5153130754212947</v>
+        <v>0.5127761157963185</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-1.65483114102164</v>
+        <v>-0.087572741938302</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6133</v>
+        <v>5243</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>金橋</t>
+          <t>乙盛-KY</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>324.0628726942797</v>
+        <v>328.1511907956772</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>23.05</v>
+        <v>109.5</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>48.20996467315496</v>
+        <v>46.8871413451367</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>12.95173212075879</v>
+        <v>15.10854183223336</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.4327375505441338</v>
+        <v>0.5153130754212947</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.0723568047073552</v>
+        <v>-1.65483114102164</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>5234</v>
+        <v>6133</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>達興材料</t>
+          <t>金橋</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>319.2198329394981</v>
+        <v>324.0628726942797</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>396</v>
+        <v>23.05</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.78955118969173</v>
+        <v>48.20996467315496</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>16.33392679344834</v>
+        <v>12.95173212075879</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.8793540348676108</v>
+        <v>0.4327375505441338</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.8179224739285411</v>
+        <v>-0.0723568047073552</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6152</v>
+        <v>5234</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>百一</t>
+          <t>達興材料</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>317.7630653696174</v>
+        <v>319.2198329394981</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>14.5</v>
+        <v>396</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>43.39972626889783</v>
+        <v>47.78955118969173</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>8.600105289912738</v>
+        <v>16.33392679344834</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.6150956201959836</v>
+        <v>0.8793540348676108</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.06655217964396989</v>
+        <v>-0.8179224739285411</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6117</v>
+        <v>6152</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>迎廣</t>
+          <t>百一</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>300.2604787107532</v>
+        <v>317.7630653696174</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>76.09999999999999</v>
+        <v>14.5</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>40.56598704800805</v>
+        <v>43.39972626889783</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>19.71387485266132</v>
+        <v>8.600105289912738</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.2401945967090524</v>
+        <v>0.6150956201959836</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.9514273092186404</v>
+        <v>-0.06655217964396989</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>4960</v>
+        <v>6117</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>誠美材</t>
+          <t>迎廣</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>293.9844239871467</v>
+        <v>300.2604787107532</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>29.1</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>40.1151956370143</v>
+        <v>40.56598704800805</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>16.58645236540448</v>
+        <v>19.71387485266132</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.7679500531169251</v>
+        <v>0.2401945967090524</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>1</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.2770693217258675</v>
+        <v>-0.9514273092186404</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>5258</v>
+        <v>4960</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>虹堡</t>
+          <t>誠美材</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>276.7280582993106</v>
+        <v>293.9844239871467</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>50.6</v>
+        <v>29.1</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>47.83180185500512</v>
+        <v>40.1151956370143</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>17.19062911115715</v>
+        <v>16.58645236540448</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.3990277096109175</v>
+        <v>0.7679500531169251</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.1561190368755657</v>
+        <v>-0.2770693217258675</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>4977</v>
+        <v>5258</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>眾達-KY</t>
+          <t>虹堡</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>275.2743837250327</v>
+        <v>276.7280582993106</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>184.5</v>
+        <v>50.6</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>45.86540242625358</v>
+        <v>47.83180185500512</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>9.588593396322535</v>
+        <v>17.19062911115715</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.5776679726960722</v>
+        <v>0.3990277096109175</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-2.259027228978113</v>
+        <v>-0.1561190368755657</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>4942</v>
+        <v>4977</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>嘉彰</t>
+          <t>眾達-KY</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>270.1745109452384</v>
+        <v>275.2743837250327</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>37.8</v>
+        <v>184.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>50.11150842603144</v>
+        <v>45.86540242625358</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>15.89483387098249</v>
+        <v>9.588593396322535</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.518109267480509</v>
+        <v>0.5776679726960722</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0055957312865507</v>
+        <v>-2.259027228978113</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6108</v>
+        <v>4942</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>競國</t>
+          <t>嘉彰</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>264.438055838805</v>
+        <v>270.1745109452384</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>19.35</v>
+        <v>37.8</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>51.46635782661846</v>
+        <v>50.11150842603144</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>12.73437280505945</v>
+        <v>15.89483387098249</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.4419367827899929</v>
+        <v>0.518109267480509</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0306715830059816</v>
+        <v>-0.0055957312865507</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>4909</v>
+        <v>6108</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>新復興</t>
+          <t>競國</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>254.348725481883</v>
+        <v>264.438055838805</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>49.85</v>
+        <v>19.35</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,16 +4368,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>43.12857169986225</v>
+        <v>51.46635782661846</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>27.6680627024909</v>
+        <v>12.73437280505945</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.5018915130328278</v>
+        <v>0.4419367827899929</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.1109707503399932</v>
+        <v>-0.0306715830059816</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>4999</v>
+        <v>4909</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>鑫禾</t>
+          <t>新復興</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>244.4647768273604</v>
+        <v>254.348725481883</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>20.65</v>
+        <v>49.85</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>48.94184188222653</v>
+        <v>43.12857169986225</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>18.24150114210192</v>
+        <v>27.6680627024909</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.5002194185220749</v>
+        <v>0.5018915130328278</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0137459676760846</v>
+        <v>0.1109707503399932</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>4905</v>
+        <v>4999</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>台聯電</t>
+          <t>鑫禾</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>240.3262143474473</v>
+        <v>244.4647768273604</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>71.90000000000001</v>
+        <v>20.65</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>40.07767414378667</v>
+        <v>48.94184188222653</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>16.59223619968574</v>
+        <v>18.24150114210192</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.3261187754974931</v>
+        <v>0.5002194185220749</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.8860393577803007</v>
+        <v>0.0137459676760846</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>5222</v>
+        <v>4905</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>全訊</t>
+          <t>台聯電</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>225.0095603044908</v>
+        <v>240.3262143474473</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>114</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>36.23763521377403</v>
+        <v>40.07767414378667</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>25.02103500373937</v>
+        <v>16.59223619968574</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.6184166819962494</v>
+        <v>0.3261187754974931</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>1</v>
@@ -4545,62 +4545,115 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.3667923616448978</v>
+        <v>-0.8860393577803007</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
+        <v>5222</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>全訊</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>225.0095603044908</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>36.23763521377403</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>25.02103500373937</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>0.6184166819962494</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>-0.3667923616448978</v>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
         <v>4994</v>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>傳奇</t>
         </is>
       </c>
-      <c r="C78" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D78" s="2" t="n">
+      <c r="C79" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D79" s="2" t="n">
         <v>173.7220565124921</v>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E79" s="2" t="n">
         <v>91.8</v>
       </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H78" s="2" t="n">
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
         <v>52.62903303779474</v>
       </c>
-      <c r="I78" s="2" t="n">
+      <c r="I79" s="2" t="n">
         <v>20.9708371145453</v>
       </c>
-      <c r="J78" s="2" t="n">
+      <c r="J79" s="2" t="n">
         <v>0.3351636028918316</v>
       </c>
-      <c r="K78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M78" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N78" s="2" t="n">
+      <c r="K79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N79" s="2" t="n">
         <v>0.8033756258927058</v>
       </c>
-      <c r="O78" s="2" t="inlineStr">
+      <c r="O79" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>

</xml_diff>